<commit_message>
Update validation hybrid data
</commit_message>
<xml_diff>
--- a/framework/data/excel/validation_hybrid.xlsx
+++ b/framework/data/excel/validation_hybrid.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\_DA\DA4\framework\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\_DA\DA4\framework\data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC87F87C-5669-4140-88E3-A51E5993C30B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBAAC9EF-9EF1-4CC1-B91D-9C818F8372DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="18240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="930" yWindow="2520" windowWidth="12450" windowHeight="13185" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestSteps" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="130">
   <si>
     <t>template_id</t>
   </si>
@@ -110,18 +110,12 @@
     <t>REALTIME_BLUR_VALIDATION</t>
   </si>
   <si>
-    <t>ClickOutside</t>
-  </si>
-  <si>
     <t>DYNAMIC_ERROR_CLEAR</t>
   </si>
   <si>
     <t>{valid_value}</t>
   </si>
   <si>
-    <t>VerifyElementNotExist</t>
-  </si>
-  <si>
     <t>Thông báo lỗi tự động biến mất ngay khi dữ liệu hợp lệ</t>
   </si>
   <si>
@@ -146,9 +140,6 @@
     <t>{phone}</t>
   </si>
   <si>
-    <t>SelectOption</t>
-  </si>
-  <si>
     <t>ddlProvince</t>
   </si>
   <si>
@@ -399,6 +390,27 @@
   </si>
   <si>
     <t>Hiển thị lỗi vượt độ dài</t>
+  </si>
+  <si>
+    <t>navigate</t>
+  </si>
+  <si>
+    <t>clickElement</t>
+  </si>
+  <si>
+    <t>setText</t>
+  </si>
+  <si>
+    <t>verifyElementNotExist</t>
+  </si>
+  <si>
+    <t>verifyText</t>
+  </si>
+  <si>
+    <t>clickOutside</t>
+  </si>
+  <si>
+    <t>selectOption</t>
   </si>
 </sst>
 </file>
@@ -1185,7 +1197,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>8</v>
@@ -1203,7 +1215,7 @@
         <v>2</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>10</v>
+        <v>124</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>18</v>
@@ -1221,7 +1233,7 @@
         <v>3</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>18</v>
@@ -1239,7 +1251,7 @@
         <v>4</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>29</v>
+        <v>128</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>18</v>
@@ -1257,7 +1269,7 @@
         <v>5</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>13</v>
+        <v>127</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>14</v>
@@ -1269,13 +1281,13 @@
     </row>
     <row r="25" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B25" s="8">
         <v>1</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>8</v>
@@ -1287,13 +1299,13 @@
     </row>
     <row r="26" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B26" s="8">
         <v>2</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>18</v>
@@ -1305,13 +1317,13 @@
     </row>
     <row r="27" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B27" s="8">
         <v>3</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>29</v>
+        <v>128</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>18</v>
@@ -1323,13 +1335,13 @@
     </row>
     <row r="28" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28" s="8">
         <v>4</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>13</v>
+        <v>127</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>14</v>
@@ -1341,49 +1353,49 @@
     </row>
     <row r="29" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" s="8">
         <v>5</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>18</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F29" s="5"/>
     </row>
     <row r="30" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="10">
         <v>6</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>32</v>
+        <v>126</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B31" s="9">
         <v>1</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>8</v>
@@ -1395,85 +1407,85 @@
     </row>
     <row r="32" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B32" s="9">
         <v>2</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F32" s="7"/>
     </row>
     <row r="33" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B33" s="9">
         <v>3</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F33" s="7"/>
     </row>
     <row r="34" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B34" s="9">
         <v>4</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>17</v>
+        <v>125</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F34" s="7"/>
     </row>
     <row r="35" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B35" s="9">
         <v>5</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>41</v>
+        <v>129</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F35" s="7"/>
     </row>
     <row r="36" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B36" s="9">
         <v>6</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>10</v>
+        <v>124</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>11</v>
@@ -1485,34 +1497,34 @@
     </row>
     <row r="37" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B37" s="9">
         <v>7</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>32</v>
+        <v>126</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B38" s="9">
         <v>8</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>13</v>
+        <v>127</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E38" s="7"/>
       <c r="F38" s="7" t="s">
@@ -1547,45 +1559,45 @@
   <sheetData>
     <row r="1" spans="1:12" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -1593,10 +1605,10 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -1607,7 +1619,7 @@
     </row>
     <row r="3" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -1615,10 +1627,10 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -1629,7 +1641,7 @@
     </row>
     <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -1637,10 +1649,10 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -1651,22 +1663,22 @@
     </row>
     <row r="5" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1677,22 +1689,22 @@
     </row>
     <row r="6" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1703,22 +1715,22 @@
     </row>
     <row r="7" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>78</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -1729,22 +1741,22 @@
     </row>
     <row r="8" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -1755,22 +1767,22 @@
     </row>
     <row r="9" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -1781,22 +1793,22 @@
     </row>
     <row r="10" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -1807,22 +1819,22 @@
     </row>
     <row r="11" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D11" s="4">
         <v>0</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -1833,22 +1845,22 @@
     </row>
     <row r="12" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D12" s="4">
         <v>150</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -1859,22 +1871,22 @@
     </row>
     <row r="13" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D13" s="4">
         <v>123</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -1885,22 +1897,22 @@
     </row>
     <row r="14" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -1911,20 +1923,20 @@
     </row>
     <row r="15" spans="1:12" ht="207" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
@@ -1935,20 +1947,20 @@
     </row>
     <row r="16" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
@@ -1959,22 +1971,22 @@
     </row>
     <row r="17" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
@@ -1985,22 +1997,22 @@
     </row>
     <row r="18" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>23</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
@@ -2011,21 +2023,21 @@
     </row>
     <row r="19" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>25</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -2035,22 +2047,22 @@
     </row>
     <row r="20" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>28</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
@@ -2061,22 +2073,22 @@
     </row>
     <row r="21" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>28</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -2087,26 +2099,26 @@
     </row>
     <row r="22" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
@@ -2115,58 +2127,58 @@
     </row>
     <row r="23" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="K23" s="4">
         <v>912345678</v>
       </c>
       <c r="L23" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="K24" s="4">
         <v>987654321</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>